<commit_message>
Update FOA set/single exports and NOT_AVAILABLE files
</commit_message>
<xml_diff>
--- a/FOA Singles/Youth-Single.xlsx
+++ b/FOA Singles/Youth-Single.xlsx
@@ -543,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC337"/>
+  <dimension ref="A1:AC336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39484,24 +39484,14 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>NOT AVAILABLE</t>
-        </is>
-      </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Gray</t>
-        </is>
-      </c>
-      <c r="C324" t="inlineStr">
-        <is>
-          <t>Gray [NOT AVAILABLE]</t>
+          <t>White/Gray</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>FM-TR452-GY</t>
+          <t>CM7467WH-TR</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -39516,134 +39506,10 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>OMNUS Trundle w/ 2 Dividers</t>
+          <t>PRIAM Trundle or Drawers</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
-        <is>
-          <t>FREE SHIPPING
-OMNUS Trundle w/ 2 Dividers adds a Transitional touch while keeping the room feeling warm and welcoming. As a youth trundle, it is designed to complement your space. Crafted from Solid Wood, Wood Veneer, Others, it is finished in Gray tones that pair easily with surrounding decor.
-Product Dimensions: 74 1 or 4" W x 40 1 or 2"D x 10 3 or 4" H
-Size: Gray [NOT AVAILABLE]
-Features
-- Made with solid wood &amp; wood veneer
-Materials: Solid Wood, Wood Veneer, Others
-Color: Gray
-Weight: 41.8 lbs</t>
-        </is>
-      </c>
-      <c r="I324" t="inlineStr">
-        <is>
-          <t>OMNUS Trundle w/ 2 Dividers Gray [NOT AVAILABLE] in Gray | GOODDEGG</t>
-        </is>
-      </c>
-      <c r="J324" t="inlineStr">
-        <is>
-          <t>The OMNUS Trundle w/ Dividers brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
-        </is>
-      </c>
-      <c r="K324" t="inlineStr">
-        <is>
-          <t>OMNUS</t>
-        </is>
-      </c>
-      <c r="L324" t="inlineStr">
-        <is>
-          <t>Trundle w/ 2 Dividers, Gray [NOT AVAILABLE]</t>
-        </is>
-      </c>
-      <c r="M324" t="inlineStr">
-        <is>
-          <t>Gray [NOT AVAILABLE] NOT AVAILABLE</t>
-        </is>
-      </c>
-      <c r="N324" t="inlineStr">
-        <is>
-          <t>Single Item</t>
-        </is>
-      </c>
-      <c r="P324" t="inlineStr">
-        <is>
-          <t>FM-TR452-GY.jpg</t>
-        </is>
-      </c>
-      <c r="Q324" t="n">
-        <v>109</v>
-      </c>
-      <c r="R324" s="1" t="n">
-        <v>109</v>
-      </c>
-      <c r="S324" t="n">
-        <v>237</v>
-      </c>
-      <c r="T324" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="U324" t="inlineStr">
-        <is>
-          <t>74 1/4"W X 40 1/2"D X 10 3/4"H</t>
-        </is>
-      </c>
-      <c r="V324" t="inlineStr">
-        <is>
-          <t>Transitional</t>
-        </is>
-      </c>
-      <c r="W324" t="inlineStr">
-        <is>
-          <t>Solid Wood, Wood Veneer, Others</t>
-        </is>
-      </c>
-      <c r="X324" t="inlineStr">
-        <is>
-          <t>Transitional,Gray,Solid Wood, Wood Veneer, Others</t>
-        </is>
-      </c>
-      <c r="Y324" t="inlineStr">
-        <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="Z324" t="n">
-        <v>79.5</v>
-      </c>
-      <c r="AA324" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="AB324" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="AC324" t="n">
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>White/Gray</t>
-        </is>
-      </c>
-      <c r="D325" t="inlineStr">
-        <is>
-          <t>CM7467WH-TR</t>
-        </is>
-      </c>
-      <c r="E325" t="inlineStr">
-        <is>
-          <t>Youth</t>
-        </is>
-      </c>
-      <c r="F325" s="24" t="inlineStr">
-        <is>
-          <t>Trundle</t>
-        </is>
-      </c>
-      <c r="G325" t="inlineStr">
-        <is>
-          <t>PRIAM Trundle or Drawers</t>
-        </is>
-      </c>
-      <c r="H325" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 Elevate your space with PRIAM Trundle or Drawers, styled in Contemporary and designed for everyday comfort. Built as a youth trundle, it pairs well with a wide range of interiors. With Solid Wood, Others and White  or  Gray tones, it blends structure and softness in one clean profile.
@@ -39657,113 +39523,113 @@
 Weight: 82.3 lbs</t>
         </is>
       </c>
-      <c r="I325" t="inlineStr">
+      <c r="I324" t="inlineStr">
         <is>
           <t>PRIAM Trundle or Drawers in White  or  Gray | GOODDEGG</t>
         </is>
       </c>
-      <c r="J325" t="inlineStr">
+      <c r="J324" t="inlineStr">
         <is>
           <t>The PRIAM Trundle or Drawers brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr">
+      <c r="K324" t="inlineStr">
         <is>
           <t>PRIAM</t>
         </is>
       </c>
-      <c r="L325" t="inlineStr">
+      <c r="L324" t="inlineStr">
         <is>
           <t>Trundle/Drawers</t>
         </is>
       </c>
-      <c r="N325" t="inlineStr">
+      <c r="N324" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P325" t="inlineStr">
+      <c r="P324" t="inlineStr">
         <is>
           <t>CM7467WH-3.jpg,FOA7467WH-TR-1-Z.jpg</t>
         </is>
       </c>
-      <c r="Q325" t="n">
+      <c r="Q324" t="n">
         <v>100</v>
       </c>
-      <c r="R325" s="2" t="n">
+      <c r="R324" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="S325" t="n">
+      <c r="S324" t="n">
         <v>270</v>
       </c>
-      <c r="T325" t="n">
+      <c r="T324" t="n">
         <v>82.3</v>
       </c>
-      <c r="U325" t="inlineStr">
+      <c r="U324" t="inlineStr">
         <is>
           <t>75 5/8"L X 40 3/4"W X 11"H</t>
         </is>
       </c>
-      <c r="V325" t="inlineStr">
+      <c r="V324" t="inlineStr">
         <is>
           <t>Contemporary</t>
         </is>
       </c>
-      <c r="W325" t="inlineStr">
+      <c r="W324" t="inlineStr">
         <is>
           <t>Solid Wood, Others</t>
         </is>
       </c>
-      <c r="X325" t="inlineStr">
+      <c r="X324" t="inlineStr">
         <is>
           <t>Contemporary,White/Gray,Solid Wood, Others,Trundle Converts to Drawers,Mattress Ready</t>
         </is>
       </c>
-      <c r="Y325" t="inlineStr">
+      <c r="Y324" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z325" t="n">
+      <c r="Z324" t="n">
         <v>82.3</v>
       </c>
-      <c r="AA325" t="n">
+      <c r="AA324" t="n">
         <v>13.1</v>
       </c>
-      <c r="AB325" t="n">
+      <c r="AB324" t="n">
         <v>5.9</v>
       </c>
-      <c r="AC325" t="n">
+      <c r="AC324" t="n">
         <v>3.7</v>
       </c>
     </row>
-    <row r="326">
-      <c r="B326" t="inlineStr">
+    <row r="325">
+      <c r="B325" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr">
+      <c r="D325" t="inlineStr">
         <is>
           <t>CM7159WH-AR-VN</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr">
+      <c r="E325" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F326" s="27" t="inlineStr">
+      <c r="F325" s="27" t="inlineStr">
         <is>
           <t>Armoire</t>
         </is>
       </c>
-      <c r="G326" t="inlineStr">
+      <c r="G325" t="inlineStr">
         <is>
           <t>DANI Armoire</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr">
+      <c r="H325" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 DANI Armoire adds a Transitional touch while keeping the room feeling warm and welcoming. As a youth armoire, it is designed to complement your space. Crafted from Solid Wood, Wood Veneer, Others, it is finished in White tones that pair easily with surrounding decor.
@@ -39775,113 +39641,113 @@
 Weight: 114.4 lbs</t>
         </is>
       </c>
-      <c r="I326" t="inlineStr">
+      <c r="I325" t="inlineStr">
         <is>
           <t>DANI Armoire in White | GOODDEGG</t>
         </is>
       </c>
-      <c r="J326" t="inlineStr">
+      <c r="J325" t="inlineStr">
         <is>
           <t>The DANI Armoire brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K326" t="inlineStr">
+      <c r="K325" t="inlineStr">
         <is>
           <t>DANI</t>
         </is>
       </c>
-      <c r="L326" t="inlineStr">
+      <c r="L325" t="inlineStr">
         <is>
           <t>Armoire</t>
         </is>
       </c>
-      <c r="N326" t="inlineStr">
+      <c r="N325" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P326" t="inlineStr">
+      <c r="P325" t="inlineStr">
         <is>
           <t>CM7159WH-AR-3.jpg,CM7159WH-AR-4.jpg,CM7159WH-AR-5.jpg,CM7159WH-AR-6.jpg,CM7159WH-AR-3-Z.jpg,CM7159WH-AR-WB.jpg</t>
         </is>
       </c>
-      <c r="Q326" t="n">
+      <c r="Q325" t="n">
         <v>289</v>
       </c>
-      <c r="R326" s="2" t="n">
+      <c r="R325" s="2" t="n">
         <v>289</v>
       </c>
-      <c r="S326" t="n">
+      <c r="S325" t="n">
         <v>717</v>
       </c>
-      <c r="T326" t="n">
+      <c r="T325" t="n">
         <v>114.4</v>
       </c>
-      <c r="U326" t="inlineStr">
+      <c r="U325" t="inlineStr">
         <is>
           <t>32 1/8"W X 16"D X 51 1/4"H</t>
         </is>
       </c>
-      <c r="V326" t="inlineStr">
+      <c r="V325" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W326" t="inlineStr">
+      <c r="W325" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X326" t="inlineStr">
+      <c r="X325" t="inlineStr">
         <is>
           <t>Transitional,White,Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="Y326" t="inlineStr">
+      <c r="Y325" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z326" t="n">
+      <c r="Z325" t="n">
         <v>35.6</v>
       </c>
-      <c r="AA326" t="n">
+      <c r="AA325" t="n">
         <v>19.5</v>
       </c>
-      <c r="AB326" t="n">
+      <c r="AB325" t="n">
         <v>56</v>
       </c>
-      <c r="AC326" t="n">
+      <c r="AC325" t="n">
         <v>22.5</v>
       </c>
     </row>
-    <row r="327">
-      <c r="B327" t="inlineStr">
+    <row r="326">
+      <c r="B326" t="inlineStr">
         <is>
           <t>Wire-Brushed Warm Gray</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr">
+      <c r="D326" t="inlineStr">
         <is>
           <t>FOA7175AR</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr">
+      <c r="E326" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F327" s="27" t="inlineStr">
+      <c r="F326" s="27" t="inlineStr">
         <is>
           <t>Armoire</t>
         </is>
       </c>
-      <c r="G327" t="inlineStr">
+      <c r="G326" t="inlineStr">
         <is>
           <t>VEVEY Armoire</t>
         </is>
       </c>
-      <c r="H327" t="inlineStr">
+      <c r="H326" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 VEVEY Armoire adds a Transitional touch while keeping the room feeling warm and welcoming. Built as a youth armoire, it pairs well with a wide range of interiors. Crafted from Solid Wood, Wood Veneer, Others, it is finished in Wire-Brushed Warm Gray tones that pair easily with surrounding decor.
@@ -39895,113 +39761,113 @@
 Weight: 156.2 lbs</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr">
+      <c r="I326" t="inlineStr">
         <is>
           <t>VEVEY Armoire in Wire-Brushed Warm Gray | GOODDEGG</t>
         </is>
       </c>
-      <c r="J327" t="inlineStr">
+      <c r="J326" t="inlineStr">
         <is>
           <t>The VEVEY Armoire brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr">
+      <c r="K326" t="inlineStr">
         <is>
           <t>VEVEY</t>
         </is>
       </c>
-      <c r="L327" t="inlineStr">
+      <c r="L326" t="inlineStr">
         <is>
           <t>Armoire</t>
         </is>
       </c>
-      <c r="N327" t="inlineStr">
+      <c r="N326" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P327" t="inlineStr">
+      <c r="P326" t="inlineStr">
         <is>
           <t>FOA7175AR-1.jpg,FOA7175-1-Z.jpg</t>
         </is>
       </c>
-      <c r="Q327" t="n">
+      <c r="Q326" t="n">
         <v>369</v>
       </c>
-      <c r="R327" s="1" t="n">
+      <c r="R326" s="1" t="n">
         <v>399</v>
       </c>
-      <c r="S327" t="n">
+      <c r="S326" t="n">
         <v>897</v>
       </c>
-      <c r="T327" t="n">
+      <c r="T326" t="n">
         <v>156.2</v>
       </c>
-      <c r="U327" t="inlineStr">
+      <c r="U326" t="inlineStr">
         <is>
           <t>40"L X 18"W X 47 3/4"H</t>
         </is>
       </c>
-      <c r="V327" t="inlineStr">
+      <c r="V326" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W327" t="inlineStr">
+      <c r="W326" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X327" t="inlineStr">
+      <c r="X326" t="inlineStr">
         <is>
           <t>Transitional,Wire-Brushed Warm Gray,Solid Wood, Wood Veneer, Others,Felt-lined Top Drawer,Round Pull Knobs,Wood Grain Texture</t>
         </is>
       </c>
-      <c r="Y327" t="inlineStr">
+      <c r="Y326" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z327" t="n">
+      <c r="Z326" t="n">
         <v>42.8</v>
       </c>
-      <c r="AA327" t="n">
+      <c r="AA326" t="n">
         <v>21</v>
       </c>
-      <c r="AB327" t="n">
+      <c r="AB326" t="n">
         <v>52.8</v>
       </c>
-      <c r="AC327" t="n">
+      <c r="AC326" t="n">
         <v>27.4</v>
       </c>
     </row>
-    <row r="328">
-      <c r="B328" t="inlineStr">
+    <row r="327">
+      <c r="B327" t="inlineStr">
         <is>
           <t>Pearl White</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr">
+      <c r="D327" t="inlineStr">
         <is>
           <t>FM72081WH-N</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr">
+      <c r="E327" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F328" s="30" t="inlineStr">
+      <c r="F327" s="30" t="inlineStr">
         <is>
           <t>Nightstand</t>
         </is>
       </c>
-      <c r="G328" t="inlineStr">
+      <c r="G327" t="inlineStr">
         <is>
           <t>LAREINA Nightstand</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr">
+      <c r="H327" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 LAREINA Nightstand brings a Contemporary look to your home with a refined, comfortable feel. This youth nightstand is made to fit naturally into the room. The Solid Rubberwood, Engineered Wood construction is complemented by Pearl White tones for a polished look.
@@ -40013,118 +39879,118 @@
 Weight: 59.97 lbs</t>
         </is>
       </c>
-      <c r="I328" t="inlineStr">
+      <c r="I327" t="inlineStr">
         <is>
           <t>LAREINA Nightstand in Pearl White | GOODDEGG</t>
         </is>
       </c>
-      <c r="J328" t="inlineStr">
+      <c r="J327" t="inlineStr">
         <is>
           <t>The LAREINA Nightstand keeps bedside essentials organized and within reach. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K328" t="inlineStr">
+      <c r="K327" t="inlineStr">
         <is>
           <t>LAREINA</t>
         </is>
       </c>
-      <c r="L328" t="inlineStr">
+      <c r="L327" t="inlineStr">
         <is>
           <t>Nightstand</t>
         </is>
       </c>
-      <c r="N328" t="inlineStr">
+      <c r="N327" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P328" t="inlineStr">
+      <c r="P327" t="inlineStr">
         <is>
           <t>FM72081WH-N-1.jpg,FM72081WH-T-1-Z.jpg,FM72081WH-N-2.jpg,FM72081WH-N-3.jpg</t>
         </is>
       </c>
-      <c r="Q328" t="n">
+      <c r="Q327" t="n">
         <v>200</v>
       </c>
-      <c r="R328" s="1" t="n">
+      <c r="R327" s="1" t="n">
         <v>210</v>
       </c>
-      <c r="S328" t="n">
+      <c r="S327" t="n">
         <v>510</v>
       </c>
-      <c r="T328" t="n">
+      <c r="T327" t="n">
         <v>59.97</v>
       </c>
-      <c r="U328" t="inlineStr">
+      <c r="U327" t="inlineStr">
         <is>
           <t>22.5"W X 17"D X 24"H</t>
         </is>
       </c>
-      <c r="V328" t="inlineStr">
+      <c r="V327" t="inlineStr">
         <is>
           <t>Contemporary</t>
         </is>
       </c>
-      <c r="W328" t="inlineStr">
+      <c r="W327" t="inlineStr">
         <is>
           <t>Solid Rubberwood, Engineered Wood</t>
         </is>
       </c>
-      <c r="X328" t="inlineStr">
+      <c r="X327" t="inlineStr">
         <is>
           <t>Contemporary,Pearl White,Solid Rubberwood, Engineered Wood,Embossed Panels,Acrylic Handles &amp; Front Legs w/ Back Metal Legs,Felt-Lined Top Drawer,Metal Glide,English Dovetails</t>
         </is>
       </c>
-      <c r="Y328" t="inlineStr">
+      <c r="Y327" t="inlineStr">
         <is>
           <t>MY</t>
         </is>
       </c>
-      <c r="Z328" t="n">
+      <c r="Z327" t="n">
         <v>25.4</v>
       </c>
-      <c r="AA328" t="n">
+      <c r="AA327" t="n">
         <v>19.6</v>
       </c>
-      <c r="AB328" t="n">
+      <c r="AB327" t="n">
         <v>24.4</v>
       </c>
-      <c r="AC328" t="n">
+      <c r="AC327" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="329">
-      <c r="B329" t="inlineStr">
+    <row r="328">
+      <c r="B328" t="inlineStr">
         <is>
           <t>Gray</t>
         </is>
       </c>
-      <c r="C329" t="inlineStr">
+      <c r="C328" t="inlineStr">
         <is>
           <t>Twin</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr">
+      <c r="D328" t="inlineStr">
         <is>
           <t>AM-BK304GY-BED</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr">
+      <c r="E328" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F329" s="32" t="inlineStr">
+      <c r="F328" s="32" t="inlineStr">
         <is>
           <t>Day Bed</t>
         </is>
       </c>
-      <c r="G329" t="inlineStr">
+      <c r="G328" t="inlineStr">
         <is>
           <t>MARINOS Captain Bed</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr">
+      <c r="H328" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 Make the room feel complete with MARINOS Captain Bed and its Rustic character. This youth day bed is made to fit naturally into the room. Finished in Gray tones, the Solid Wood, Others build balances durability with visual appeal.
@@ -40139,114 +40005,114 @@
 Weight: 171 lbs</t>
         </is>
       </c>
-      <c r="I329" t="inlineStr">
+      <c r="I328" t="inlineStr">
         <is>
           <t>MARINOS Captain Bed Twin in Gray | GOODDEGG</t>
         </is>
       </c>
-      <c r="J329" t="inlineStr">
+      <c r="J328" t="inlineStr">
         <is>
           <t>The MARINOS Captain Bed creates a restful centerpiece for the bedroom. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr">
+      <c r="K328" t="inlineStr">
         <is>
           <t>MARINOS</t>
         </is>
       </c>
-      <c r="L329" t="inlineStr">
+      <c r="L328" t="inlineStr">
         <is>
           <t>Twin Captain Bed</t>
         </is>
       </c>
-      <c r="N329" t="inlineStr">
+      <c r="N328" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="O329" t="inlineStr">
+      <c r="O328" t="inlineStr">
         <is>
           <t>AM-BK304GY-1, AM-BK304GY-2, AM-BK304GY-3, AM-BK304GY-4, AM-BK304GY-5, AM-SL109-T</t>
         </is>
       </c>
-      <c r="P329" t="inlineStr">
+      <c r="P328" t="inlineStr">
         <is>
           <t>AM-BK304GY-1.jpg</t>
         </is>
       </c>
-      <c r="Q329" t="n">
+      <c r="Q328" t="n">
         <v>449</v>
       </c>
-      <c r="R329" s="1" t="n">
+      <c r="R328" s="1" t="n">
         <v>449</v>
       </c>
-      <c r="S329" t="n">
+      <c r="S328" t="n">
         <v>1347</v>
       </c>
-      <c r="T329" t="n">
+      <c r="T328" t="n">
         <v>171</v>
       </c>
-      <c r="U329" t="inlineStr">
+      <c r="U328" t="inlineStr">
         <is>
           <t>78"W X 41"D X 34"H</t>
         </is>
       </c>
-      <c r="V329" t="inlineStr">
+      <c r="V328" t="inlineStr">
         <is>
           <t>Rustic</t>
         </is>
       </c>
-      <c r="W329" t="inlineStr">
+      <c r="W328" t="inlineStr">
         <is>
           <t>Solid Wood, Others</t>
         </is>
       </c>
-      <c r="X329" t="inlineStr">
+      <c r="X328" t="inlineStr">
         <is>
           <t>Rustic,Gray,Solid Wood, Others,Fits up to 6" Mattress,Large Underbed Drawers,Bronze Round Knobs,Brazilian Pine Construction</t>
         </is>
       </c>
-      <c r="Y329" t="inlineStr">
+      <c r="Y328" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="AC329" t="n">
+      <c r="AC328" t="n">
         <v>22.3</v>
       </c>
     </row>
-    <row r="330">
-      <c r="B330" t="inlineStr">
+    <row r="329">
+      <c r="B329" t="inlineStr">
         <is>
           <t>Mahogany</t>
         </is>
       </c>
-      <c r="C330" t="inlineStr">
+      <c r="C329" t="inlineStr">
         <is>
           <t>Twin</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr">
+      <c r="D329" t="inlineStr">
         <is>
           <t>AM-BK304MH-BED</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr">
+      <c r="E329" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F330" s="32" t="inlineStr">
+      <c r="F329" s="32" t="inlineStr">
         <is>
           <t>Day Bed</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr">
+      <c r="G329" t="inlineStr">
         <is>
           <t>MARINOS Captain Bed</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr">
+      <c r="H329" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 MARINOS Captain Bed brings a Rustic look to your home with a refined, comfortable feel. Built as a youth day bed, it pairs well with a wide range of interiors. The Solid Wood, Others construction is complemented by Mahogany tones for a polished look.
@@ -40261,109 +40127,109 @@
 Weight: 171 lbs</t>
         </is>
       </c>
-      <c r="I330" t="inlineStr">
+      <c r="I329" t="inlineStr">
         <is>
           <t>MARINOS Captain Bed Twin in Mahogany | GOODDEGG</t>
         </is>
       </c>
-      <c r="J330" t="inlineStr">
+      <c r="J329" t="inlineStr">
         <is>
           <t>The MARINOS Captain Bed creates a restful centerpiece for the bedroom. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K330" t="inlineStr">
+      <c r="K329" t="inlineStr">
         <is>
           <t>MARINOS</t>
         </is>
       </c>
-      <c r="L330" t="inlineStr">
+      <c r="L329" t="inlineStr">
         <is>
           <t>Twin Captain Bed</t>
         </is>
       </c>
-      <c r="N330" t="inlineStr">
+      <c r="N329" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="O330" t="inlineStr">
+      <c r="O329" t="inlineStr">
         <is>
           <t>AM-BK304MH-1, AM-BK304MH-2, AM-BK304MH-3, AM-BK304MH-4, AM-BK304MH-5, AM-SL109-T</t>
         </is>
       </c>
-      <c r="P330" t="inlineStr">
+      <c r="P329" t="inlineStr">
         <is>
           <t>AM-BK304MH-1.jpg</t>
         </is>
       </c>
-      <c r="Q330" t="n">
+      <c r="Q329" t="n">
         <v>449</v>
       </c>
-      <c r="R330" s="1" t="n">
+      <c r="R329" s="1" t="n">
         <v>449</v>
       </c>
-      <c r="S330" t="n">
+      <c r="S329" t="n">
         <v>1347</v>
       </c>
-      <c r="T330" t="n">
+      <c r="T329" t="n">
         <v>171</v>
       </c>
-      <c r="U330" t="inlineStr">
+      <c r="U329" t="inlineStr">
         <is>
           <t>78"W X 41"D X 34"H</t>
         </is>
       </c>
-      <c r="V330" t="inlineStr">
+      <c r="V329" t="inlineStr">
         <is>
           <t>Rustic</t>
         </is>
       </c>
-      <c r="W330" t="inlineStr">
+      <c r="W329" t="inlineStr">
         <is>
           <t>Solid Wood, Others</t>
         </is>
       </c>
-      <c r="X330" t="inlineStr">
+      <c r="X329" t="inlineStr">
         <is>
           <t>Rustic,Mahogany,Solid Wood, Others,Fits up to 6" Mattress,Large Underbed Drawers,Black Round Knobs,Brazilian Pine Construction</t>
         </is>
       </c>
-      <c r="Y330" t="inlineStr">
+      <c r="Y329" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="AC330" t="n">
+      <c r="AC329" t="n">
         <v>22.3</v>
       </c>
     </row>
-    <row r="331">
-      <c r="B331" t="inlineStr">
+    <row r="330">
+      <c r="B330" t="inlineStr">
         <is>
           <t>Cherry</t>
         </is>
       </c>
-      <c r="D331" t="inlineStr">
+      <c r="D330" t="inlineStr">
         <is>
           <t>CM7905CH-DK</t>
         </is>
       </c>
-      <c r="E331" t="inlineStr">
+      <c r="E330" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F331" s="34" t="inlineStr">
+      <c r="F330" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G331" t="inlineStr">
+      <c r="G330" t="inlineStr">
         <is>
           <t>OMNUS Desk</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr">
+      <c r="H330" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 OMNUS Desk adds a Transitional touch while keeping the room feeling warm and welcoming. Built as a youth desk, it pairs well with a wide range of interiors. Crafted from Solid Wood, Wood Veneer, Others, it is finished in Cherry tones that pair easily with surrounding decor.
@@ -40375,113 +40241,113 @@
 Weight: 88.2 lbs</t>
         </is>
       </c>
-      <c r="I331" t="inlineStr">
+      <c r="I330" t="inlineStr">
         <is>
           <t>OMNUS Desk in Cherry | GOODDEGG</t>
         </is>
       </c>
-      <c r="J331" t="inlineStr">
+      <c r="J330" t="inlineStr">
         <is>
           <t>The OMNUS Desk creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr">
+      <c r="K330" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L331" t="inlineStr">
+      <c r="L330" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="N331" t="inlineStr">
+      <c r="N330" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P331" t="inlineStr">
+      <c r="P330" t="inlineStr">
         <is>
           <t>CM7905CH-DK.jpg,CM7905CH-DK+HC-tray.jpg</t>
         </is>
       </c>
-      <c r="Q331" t="n">
+      <c r="Q330" t="n">
         <v>289</v>
       </c>
-      <c r="R331" s="1" t="n">
+      <c r="R330" s="1" t="n">
         <v>312</v>
       </c>
-      <c r="S331" t="n">
+      <c r="S330" t="n">
         <v>690</v>
       </c>
-      <c r="T331" t="n">
+      <c r="T330" t="n">
         <v>88.2</v>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="U330" t="inlineStr">
         <is>
           <t>48"W X 20"D X 32"H</t>
         </is>
       </c>
-      <c r="V331" t="inlineStr">
+      <c r="V330" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W331" t="inlineStr">
+      <c r="W330" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X331" t="inlineStr">
+      <c r="X330" t="inlineStr">
         <is>
           <t>Transitional,Cherry,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y331" t="inlineStr">
+      <c r="Y330" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z331" t="n">
+      <c r="Z330" t="n">
         <v>23.5</v>
       </c>
-      <c r="AA331" t="n">
+      <c r="AA330" t="n">
         <v>51.5</v>
       </c>
-      <c r="AB331" t="n">
+      <c r="AB330" t="n">
         <v>36.5</v>
       </c>
-      <c r="AC331" t="n">
+      <c r="AC330" t="n">
         <v>25.6</v>
       </c>
     </row>
-    <row r="332">
-      <c r="B332" t="inlineStr">
+    <row r="331">
+      <c r="B331" t="inlineStr">
         <is>
           <t>Dark Walnut</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr">
+      <c r="D331" t="inlineStr">
         <is>
           <t>CM7905EXP-DK</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr">
+      <c r="E331" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F332" s="34" t="inlineStr">
+      <c r="F331" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G332" t="inlineStr">
+      <c r="G331" t="inlineStr">
         <is>
           <t>OMNUS Desk</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr">
+      <c r="H331" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 Make the room feel complete with OMNUS Desk and its Transitional character. As a youth desk, it is designed to complement your space. Finished in Dark Walnut tones, the Solid Wood, Wood Veneer, Others build balances durability with visual appeal.
@@ -40493,113 +40359,113 @@
 Weight: 88.2 lbs</t>
         </is>
       </c>
-      <c r="I332" t="inlineStr">
+      <c r="I331" t="inlineStr">
         <is>
           <t>OMNUS Desk in Dark Walnut | GOODDEGG</t>
         </is>
       </c>
-      <c r="J332" t="inlineStr">
+      <c r="J331" t="inlineStr">
         <is>
           <t>The OMNUS Desk creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K332" t="inlineStr">
+      <c r="K331" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L332" t="inlineStr">
+      <c r="L331" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="N332" t="inlineStr">
+      <c r="N331" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P332" t="inlineStr">
+      <c r="P331" t="inlineStr">
         <is>
           <t>CM7905EXP-DK.jpg,CM7905EXP-DK+HC.jpg</t>
         </is>
       </c>
-      <c r="Q332" t="n">
+      <c r="Q331" t="n">
         <v>289</v>
       </c>
-      <c r="R332" s="2" t="n">
+      <c r="R331" s="2" t="n">
         <v>289</v>
       </c>
-      <c r="S332" t="n">
+      <c r="S331" t="n">
         <v>657</v>
       </c>
-      <c r="T332" t="n">
+      <c r="T331" t="n">
         <v>88.2</v>
       </c>
-      <c r="U332" t="inlineStr">
+      <c r="U331" t="inlineStr">
         <is>
           <t>48"W X 20"D X 32"H</t>
         </is>
       </c>
-      <c r="V332" t="inlineStr">
+      <c r="V331" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W332" t="inlineStr">
+      <c r="W331" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X332" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>Transitional,Dark Walnut,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y332" t="inlineStr">
+      <c r="Y331" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z332" t="n">
+      <c r="Z331" t="n">
         <v>51</v>
       </c>
-      <c r="AA332" t="n">
+      <c r="AA331" t="n">
         <v>23</v>
       </c>
-      <c r="AB332" t="n">
+      <c r="AB331" t="n">
         <v>34.3</v>
       </c>
-      <c r="AC332" t="n">
+      <c r="AC331" t="n">
         <v>23.2</v>
       </c>
     </row>
-    <row r="333">
-      <c r="B333" t="inlineStr">
+    <row r="332">
+      <c r="B332" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr">
+      <c r="D332" t="inlineStr">
         <is>
           <t>CM7905WH-DK</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr">
+      <c r="E332" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F333" s="34" t="inlineStr">
+      <c r="F332" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G333" t="inlineStr">
+      <c r="G332" t="inlineStr">
         <is>
           <t>OMNUS Desk</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr">
+      <c r="H332" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 OMNUS Desk brings a Transitional look to your home with a refined, comfortable feel. This youth desk is made to fit naturally into the room. The Solid Wood, Wood Veneer, Others construction is complemented by White tones for a polished look.
@@ -40611,113 +40477,113 @@
 Weight: 88.2 lbs</t>
         </is>
       </c>
-      <c r="I333" t="inlineStr">
+      <c r="I332" t="inlineStr">
         <is>
           <t>OMNUS Desk in White | GOODDEGG</t>
         </is>
       </c>
-      <c r="J333" t="inlineStr">
+      <c r="J332" t="inlineStr">
         <is>
           <t>The OMNUS Desk creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr">
+      <c r="K332" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L333" t="inlineStr">
+      <c r="L332" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="N333" t="inlineStr">
+      <c r="N332" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P333" t="inlineStr">
+      <c r="P332" t="inlineStr">
         <is>
           <t>CM7905WH-DK.jpg</t>
         </is>
       </c>
-      <c r="Q333" t="n">
+      <c r="Q332" t="n">
         <v>289</v>
       </c>
-      <c r="R333" s="2" t="n">
+      <c r="R332" s="2" t="n">
         <v>289</v>
       </c>
-      <c r="S333" t="n">
+      <c r="S332" t="n">
         <v>657</v>
       </c>
-      <c r="T333" t="n">
+      <c r="T332" t="n">
         <v>88.2</v>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="U332" t="inlineStr">
         <is>
           <t>48"W X 20"D X 32"H</t>
         </is>
       </c>
-      <c r="V333" t="inlineStr">
+      <c r="V332" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W333" t="inlineStr">
+      <c r="W332" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X333" t="inlineStr">
+      <c r="X332" t="inlineStr">
         <is>
           <t>Transitional,White,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y333" t="inlineStr">
+      <c r="Y332" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z333" t="n">
+      <c r="Z332" t="n">
         <v>23.5</v>
       </c>
-      <c r="AA333" t="n">
+      <c r="AA332" t="n">
         <v>51.5</v>
       </c>
-      <c r="AB333" t="n">
+      <c r="AB332" t="n">
         <v>36.5</v>
       </c>
-      <c r="AC333" t="n">
+      <c r="AC332" t="n">
         <v>25.6</v>
       </c>
     </row>
-    <row r="334">
-      <c r="B334" t="inlineStr">
+    <row r="333">
+      <c r="B333" t="inlineStr">
         <is>
           <t>Cherry</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr">
+      <c r="D333" t="inlineStr">
         <is>
           <t>CM7905CH-HC</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr">
+      <c r="E333" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F334" s="34" t="inlineStr">
+      <c r="F333" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G334" t="inlineStr">
+      <c r="G333" t="inlineStr">
         <is>
           <t>OMNUS Hutch</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr">
+      <c r="H333" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 OMNUS Hutch brings a Transitional look to your home with a refined, comfortable feel. Built as a youth desk, it pairs well with a wide range of interiors. The Solid Wood, Wood Veneer, Others construction is complemented by Cherry tones for a polished look.
@@ -40729,113 +40595,113 @@
 Weight: 29.76 lbs</t>
         </is>
       </c>
-      <c r="I334" t="inlineStr">
+      <c r="I333" t="inlineStr">
         <is>
           <t>OMNUS Hutch in Cherry | GOODDEGG</t>
         </is>
       </c>
-      <c r="J334" t="inlineStr">
+      <c r="J333" t="inlineStr">
         <is>
           <t>The OMNUS Hutch creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K334" t="inlineStr">
+      <c r="K333" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L334" t="inlineStr">
+      <c r="L333" t="inlineStr">
         <is>
           <t>Hutch</t>
         </is>
       </c>
-      <c r="N334" t="inlineStr">
+      <c r="N333" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P334" t="inlineStr">
+      <c r="P333" t="inlineStr">
         <is>
           <t>CM7905CH-HC.jpg,CM7903CH-Z.jpg</t>
         </is>
       </c>
-      <c r="Q334" t="n">
+      <c r="Q333" t="n">
         <v>110</v>
       </c>
-      <c r="R334" s="1" t="n">
+      <c r="R333" s="1" t="n">
         <v>119</v>
       </c>
-      <c r="S334" t="n">
+      <c r="S333" t="n">
         <v>270</v>
       </c>
-      <c r="T334" t="n">
+      <c r="T333" t="n">
         <v>29.76</v>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="U333" t="inlineStr">
         <is>
           <t>46"W X 12"D X 24"H</t>
         </is>
       </c>
-      <c r="V334" t="inlineStr">
+      <c r="V333" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W334" t="inlineStr">
+      <c r="W333" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X334" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>Transitional,Cherry,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y334" t="inlineStr">
+      <c r="Y333" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z334" t="n">
+      <c r="Z333" t="n">
         <v>25.8</v>
       </c>
-      <c r="AA334" t="n">
+      <c r="AA333" t="n">
         <v>49</v>
       </c>
-      <c r="AB334" t="n">
+      <c r="AB333" t="n">
         <v>12.8</v>
       </c>
-      <c r="AC334" t="n">
+      <c r="AC333" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
-    <row r="335">
-      <c r="B335" t="inlineStr">
+    <row r="334">
+      <c r="B334" t="inlineStr">
         <is>
           <t>Dark Walnut</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
+      <c r="D334" t="inlineStr">
         <is>
           <t>CM7905EXP-HC</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr">
+      <c r="E334" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F335" s="34" t="inlineStr">
+      <c r="F334" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G335" t="inlineStr">
+      <c r="G334" t="inlineStr">
         <is>
           <t>OMNUS Hutch</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr">
+      <c r="H334" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 Elevate your space with OMNUS Hutch, styled in Transitional and designed for everyday comfort. As a youth desk, it is designed to complement your space. With Solid Wood, Wood Veneer, Others and Dark Walnut tones, it blends structure and softness in one clean profile.
@@ -40847,113 +40713,113 @@
 Weight: 27.6 lbs</t>
         </is>
       </c>
-      <c r="I335" t="inlineStr">
+      <c r="I334" t="inlineStr">
         <is>
           <t>OMNUS Hutch in Dark Walnut | GOODDEGG</t>
         </is>
       </c>
-      <c r="J335" t="inlineStr">
+      <c r="J334" t="inlineStr">
         <is>
           <t>The OMNUS Hutch creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K335" t="inlineStr">
+      <c r="K334" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L335" t="inlineStr">
+      <c r="L334" t="inlineStr">
         <is>
           <t>Hutch</t>
         </is>
       </c>
-      <c r="N335" t="inlineStr">
+      <c r="N334" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P335" t="inlineStr">
+      <c r="P334" t="inlineStr">
         <is>
           <t>CM7905EXP-HC.jpg</t>
         </is>
       </c>
-      <c r="Q335" t="n">
+      <c r="Q334" t="n">
         <v>110</v>
       </c>
-      <c r="R335" s="2" t="n">
+      <c r="R334" s="2" t="n">
         <v>110</v>
       </c>
-      <c r="S335" t="n">
+      <c r="S334" t="n">
         <v>270</v>
       </c>
-      <c r="T335" t="n">
+      <c r="T334" t="n">
         <v>27.6</v>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="U334" t="inlineStr">
         <is>
           <t>46"W X 12"D X 24"H</t>
         </is>
       </c>
-      <c r="V335" t="inlineStr">
+      <c r="V334" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W335" t="inlineStr">
+      <c r="W334" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X335" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>Transitional,Dark Walnut,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y335" t="inlineStr">
+      <c r="Y334" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z335" t="n">
+      <c r="Z334" t="n">
         <v>48.1</v>
       </c>
-      <c r="AA335" t="n">
+      <c r="AA334" t="n">
         <v>25</v>
       </c>
-      <c r="AB335" t="n">
+      <c r="AB334" t="n">
         <v>12.5</v>
       </c>
-      <c r="AC335" t="n">
+      <c r="AC334" t="n">
         <v>8.699999999999999</v>
       </c>
     </row>
-    <row r="336">
-      <c r="B336" t="inlineStr">
+    <row r="335">
+      <c r="B335" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>CM7905WH-HC</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr">
+      <c r="E335" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F336" s="34" t="inlineStr">
+      <c r="F335" s="34" t="inlineStr">
         <is>
           <t>Desk</t>
         </is>
       </c>
-      <c r="G336" t="inlineStr">
+      <c r="G335" t="inlineStr">
         <is>
           <t>OMNUS Hutch</t>
         </is>
       </c>
-      <c r="H336" t="inlineStr">
+      <c r="H335" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 OMNUS Hutch adds a Transitional touch while keeping the room feeling warm and welcoming. This youth desk is made to fit naturally into the room. Crafted from Solid Wood, Wood Veneer, Others, it is finished in White tones that pair easily with surrounding decor.
@@ -40965,113 +40831,113 @@
 Weight: 27.6 lbs</t>
         </is>
       </c>
-      <c r="I336" t="inlineStr">
+      <c r="I335" t="inlineStr">
         <is>
           <t>OMNUS Hutch in White | GOODDEGG</t>
         </is>
       </c>
-      <c r="J336" t="inlineStr">
+      <c r="J335" t="inlineStr">
         <is>
           <t>The OMNUS Hutch creates a focused workspace for daily tasks. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr">
+      <c r="K335" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L336" t="inlineStr">
+      <c r="L335" t="inlineStr">
         <is>
           <t>Hutch</t>
         </is>
       </c>
-      <c r="N336" t="inlineStr">
+      <c r="N335" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P336" t="inlineStr">
+      <c r="P335" t="inlineStr">
         <is>
           <t>CM7905WH-HC.jpg,CM7902WH.jpg</t>
         </is>
       </c>
-      <c r="Q336" t="n">
+      <c r="Q335" t="n">
         <v>110</v>
       </c>
-      <c r="R336" s="2" t="n">
+      <c r="R335" s="2" t="n">
         <v>110</v>
       </c>
-      <c r="S336" t="n">
+      <c r="S335" t="n">
         <v>270</v>
       </c>
-      <c r="T336" t="n">
+      <c r="T335" t="n">
         <v>27.6</v>
       </c>
-      <c r="U336" t="inlineStr">
+      <c r="U335" t="inlineStr">
         <is>
           <t>46"W X 12"D X 24"H</t>
         </is>
       </c>
-      <c r="V336" t="inlineStr">
+      <c r="V335" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W336" t="inlineStr">
+      <c r="W335" t="inlineStr">
         <is>
           <t>Solid Wood, Wood Veneer, Others</t>
         </is>
       </c>
-      <c r="X336" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>Transitional,White,Solid Wood, Wood Veneer, Others,Match w, Various Youth Beds</t>
         </is>
       </c>
-      <c r="Y336" t="inlineStr">
+      <c r="Y335" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z336" t="n">
+      <c r="Z335" t="n">
         <v>25.8</v>
       </c>
-      <c r="AA336" t="n">
+      <c r="AA335" t="n">
         <v>49</v>
       </c>
-      <c r="AB336" t="n">
+      <c r="AB335" t="n">
         <v>12.8</v>
       </c>
-      <c r="AC336" t="n">
+      <c r="AC335" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
-    <row r="337">
-      <c r="B337" t="inlineStr">
+    <row r="336">
+      <c r="B336" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D336" t="inlineStr">
         <is>
           <t>CM-SR452-WH</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E336" t="inlineStr">
         <is>
           <t>Youth</t>
         </is>
       </c>
-      <c r="F337" s="37" t="inlineStr">
+      <c r="F336" s="37" t="inlineStr">
         <is>
           <t>Shelf/Storage</t>
         </is>
       </c>
-      <c r="G337" t="inlineStr">
+      <c r="G336" t="inlineStr">
         <is>
           <t>OMNUS Underbed Storage w/ Sliding Doors</t>
         </is>
       </c>
-      <c r="H337" t="inlineStr">
+      <c r="H336" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 Make the room feel complete with OMNUS Underbed Storage w/ Sliding Doors and its Transitional character. This youth shelf or storage is made to fit naturally into the room. Finished in White tones, the Solid Wood, Others build balances durability with visual appeal.
@@ -41083,83 +40949,83 @@
 Weight: 52.8 lbs</t>
         </is>
       </c>
-      <c r="I337" t="inlineStr">
+      <c r="I336" t="inlineStr">
         <is>
           <t>OMNUS Underbed Storage w/ Sliding Doors in White | GOODDEGG</t>
         </is>
       </c>
-      <c r="J337" t="inlineStr">
+      <c r="J336" t="inlineStr">
         <is>
           <t>OMNUS Underbed Storage w/ Sliding Doors organizes and displays your essentials with ease. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr">
+      <c r="K336" t="inlineStr">
         <is>
           <t>OMNUS</t>
         </is>
       </c>
-      <c r="L337" t="inlineStr">
+      <c r="L336" t="inlineStr">
         <is>
           <t>Underbed Storage w/ Sliding Doors</t>
         </is>
       </c>
-      <c r="N337" t="inlineStr">
+      <c r="N336" t="inlineStr">
         <is>
           <t>Single Item</t>
         </is>
       </c>
-      <c r="P337" t="inlineStr">
+      <c r="P336" t="inlineStr">
         <is>
           <t>CM-SR452-WH-1-Z.jpg,CM-SR452-WH-2.jpg</t>
         </is>
       </c>
-      <c r="Q337" t="n">
+      <c r="Q336" t="n">
         <v>160</v>
       </c>
-      <c r="R337" s="2" t="n">
+      <c r="R336" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="S337" t="n">
+      <c r="S336" t="n">
         <v>450</v>
       </c>
-      <c r="T337" t="n">
+      <c r="T336" t="n">
         <v>52.8</v>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="U336" t="inlineStr">
         <is>
           <t>75 1/2"L X15 3/4 "W X 10 1/2"H</t>
         </is>
       </c>
-      <c r="V337" t="inlineStr">
+      <c r="V336" t="inlineStr">
         <is>
           <t>Transitional</t>
         </is>
       </c>
-      <c r="W337" t="inlineStr">
+      <c r="W336" t="inlineStr">
         <is>
           <t>Solid Wood, Others</t>
         </is>
       </c>
-      <c r="X337" t="inlineStr">
+      <c r="X336" t="inlineStr">
         <is>
           <t>Transitional,White,Solid Wood, Others,Storage with Sliding Doors</t>
         </is>
       </c>
-      <c r="Y337" t="inlineStr">
+      <c r="Y336" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="Z337" t="n">
+      <c r="Z336" t="n">
         <v>79.5</v>
       </c>
-      <c r="AA337" t="n">
+      <c r="AA336" t="n">
         <v>19.3</v>
       </c>
-      <c r="AB337" t="n">
+      <c r="AB336" t="n">
         <v>12</v>
       </c>
-      <c r="AC337" t="n">
+      <c r="AC336" t="n">
         <v>10.6</v>
       </c>
     </row>

</xml_diff>